<commit_message>
Update to v1.1.2: add journal, receipt PNG/PDF export, multi-currency totals, UI refresh, and verification suite
</commit_message>
<xml_diff>
--- a/tests/filtered.xlsx
+++ b/tests/filtered.xlsx
@@ -70,7 +70,7 @@
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="7" width="24" customWidth="1"/>
-    <col min="8" max="10" width="19" customWidth="1"/>
+    <col min="8" max="11" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -121,7 +121,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">روپیہ</t>
+          <t xml:space="preserve">روپیہ (PKR)</t>
         </is>
       </c>
     </row>
@@ -172,7 +172,7 @@
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">کل مجموعہ</t>
+          <t xml:space="preserve">کل مجموعہ حساب</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">

</xml_diff>